<commit_message>
Correct no callback in admin routes put route
</commit_message>
<xml_diff>
--- a/test/Assets/Lists.xlsx
+++ b/test/Assets/Lists.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ian/Documents/naap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ian/Documents/Projects/nap/test/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CDB33B4-2D5F-924F-9FF5-2F4247E76F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F305C9-1DCD-2242-8DF0-9CA2A7CBDF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3580" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{C06FBE5E-17A7-D341-AC99-42140C686358}"/>
+    <workbookView xWindow="3580" yWindow="2160" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{C06FBE5E-17A7-D341-AC99-42140C686358}"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="74">
   <si>
     <t>company</t>
   </si>
@@ -336,9 +336,6 @@
   </si>
   <si>
     <t>     INTERCOMPANY AND RELATED PARTY ACCOUNTS</t>
-  </si>
-  <si>
-    <t>Description</t>
   </si>
   <si>
     <t>company_id</t>
@@ -788,7 +785,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -797,16 +794,16 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
@@ -815,7 +812,7 @@
         <v>6</v>
       </c>
       <c r="J1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K1" t="s">
         <v>8</v>
@@ -823,101 +820,101 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" t="s">
         <v>63</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>64</v>
-      </c>
-      <c r="I2" t="s">
-        <v>65</v>
       </c>
       <c r="J2">
         <v>30342</v>
       </c>
       <c r="K2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s">
-        <v>58</v>
-      </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
       <c r="F3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" t="s">
         <v>63</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>64</v>
-      </c>
-      <c r="I3" t="s">
-        <v>65</v>
       </c>
       <c r="J3">
         <v>30342</v>
       </c>
       <c r="K3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" t="s">
         <v>67</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>68</v>
-      </c>
-      <c r="D4" t="s">
-        <v>69</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
       </c>
       <c r="F4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" t="s">
         <v>70</v>
       </c>
-      <c r="G4" t="s">
-        <v>71</v>
-      </c>
       <c r="H4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" t="s">
         <v>64</v>
-      </c>
-      <c r="I4" t="s">
-        <v>65</v>
       </c>
       <c r="J4">
         <v>30328</v>
       </c>
       <c r="K4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -936,10 +933,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B1" t="s">
-        <v>49</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1025,13 +1022,13 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G1" t="s">
         <v>9</v>
@@ -1090,7 +1087,7 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
         <v>5</v>
@@ -1136,7 +1133,7 @@
         <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F1" t="s">
         <v>20</v>
@@ -1199,7 +1196,7 @@
         <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I1" t="s">
         <v>1</v>
@@ -1258,7 +1255,7 @@
         <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
complete proyotype controllers and models for GL
</commit_message>
<xml_diff>
--- a/test/Assets/Lists.xlsx
+++ b/test/Assets/Lists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ian/Documents/Projects/nap/test/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F305C9-1DCD-2242-8DF0-9CA2A7CBDF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECD41A2-9D7F-6B4F-BF16-9755AD532B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3580" yWindow="2160" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{C06FBE5E-17A7-D341-AC99-42140C686358}"/>
+    <workbookView xWindow="4280" yWindow="4280" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{C06FBE5E-17A7-D341-AC99-42140C686358}"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Customers" sheetId="5" r:id="rId6"/>
     <sheet name="Employees" sheetId="6" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="210">
   <si>
     <t>company</t>
   </si>
@@ -74,174 +74,6 @@
     <t>account</t>
   </si>
   <si>
-    <r>
-      <t>1.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ASSETS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>2.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>LIABILITIES</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>3.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>EQUITY</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>4.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>REVENUE/INCOME</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>5.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>EXPENSES</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>6.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>OTHER (NON-OPERATING) INCOME AND EXPENSES</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>7.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>INTERCOMPANY AND RELATED PARTY ACCOUNTS</t>
-    </r>
-  </si>
-  <si>
     <t>vendor_id</t>
   </si>
   <si>
@@ -317,27 +149,6 @@
     <t>notes</t>
   </si>
   <si>
-    <t>     ASSETS</t>
-  </si>
-  <si>
-    <t>     LIABILITIES</t>
-  </si>
-  <si>
-    <t>     EQUITY</t>
-  </si>
-  <si>
-    <t>     REVENUE/INCOME</t>
-  </si>
-  <si>
-    <t>     EXPENSES</t>
-  </si>
-  <si>
-    <t>     OTHER (NON-OPERATING) INCOME AND EXPENSES</t>
-  </si>
-  <si>
-    <t>     INTERCOMPANY AND RELATED PARTY ACCOUNTS</t>
-  </si>
-  <si>
     <t>company_id</t>
   </si>
   <si>
@@ -411,25 +222,469 @@
   </si>
   <si>
     <t>tax_id</t>
+  </si>
+  <si>
+    <t>INCOME</t>
+  </si>
+  <si>
+    <t>LIABILITIES</t>
+  </si>
+  <si>
+    <t>EQUITY</t>
+  </si>
+  <si>
+    <t>EXPENSES</t>
+  </si>
+  <si>
+    <t>OTHER (NON-OPERATING) INCOME AND EXPENSES</t>
+  </si>
+  <si>
+    <t>ASSETS</t>
+  </si>
+  <si>
+    <t>INTERCOMPANY ACCOUNTS</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>WIP</t>
+  </si>
+  <si>
+    <t>Property, Plant and Equipment</t>
+  </si>
+  <si>
+    <t>Credit Cards</t>
+  </si>
+  <si>
+    <t>Loans</t>
+  </si>
+  <si>
+    <t>Capital Account</t>
+  </si>
+  <si>
+    <t>COGS</t>
+  </si>
+  <si>
+    <t>Direct Expenses</t>
+  </si>
+  <si>
+    <t>Indirect Expenses</t>
+  </si>
+  <si>
+    <t>Payroll</t>
+  </si>
+  <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>1.3</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>2.2</t>
+  </si>
+  <si>
+    <t>2.4</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>5.1</t>
+  </si>
+  <si>
+    <t>5.2</t>
+  </si>
+  <si>
+    <t>5.3</t>
+  </si>
+  <si>
+    <t>5.6</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>1.1.1000</t>
+  </si>
+  <si>
+    <t>Company Cash Account 1</t>
+  </si>
+  <si>
+    <t>1.1.1010</t>
+  </si>
+  <si>
+    <t>Company Cash Account 2</t>
+  </si>
+  <si>
+    <t>1.1.1020</t>
+  </si>
+  <si>
+    <t>Company Cash Account 3</t>
+  </si>
+  <si>
+    <t>1.1.1990</t>
+  </si>
+  <si>
+    <t>Cash - Clearing</t>
+  </si>
+  <si>
+    <t>1.2.2000</t>
+  </si>
+  <si>
+    <t>Accounts Receivable</t>
+  </si>
+  <si>
+    <t>1.3.3000</t>
+  </si>
+  <si>
+    <t>WIP - Land</t>
+  </si>
+  <si>
+    <t>1.3.3100</t>
+  </si>
+  <si>
+    <t>WIP - Vertical</t>
+  </si>
+  <si>
+    <t>1.4.4000</t>
+  </si>
+  <si>
+    <t>Options on Land</t>
+  </si>
+  <si>
+    <t>1.5.5000</t>
+  </si>
+  <si>
+    <t>Office Furniture and Equipment</t>
+  </si>
+  <si>
+    <t>1.5.5010</t>
+  </si>
+  <si>
+    <t>Model Furniture and Equipment</t>
+  </si>
+  <si>
+    <t>1.5.5020</t>
+  </si>
+  <si>
+    <t>Accumulated Depreciation</t>
+  </si>
+  <si>
+    <t>2.1.1000</t>
+  </si>
+  <si>
+    <t>Accounts Payable</t>
+  </si>
+  <si>
+    <t>2.2.2000</t>
+  </si>
+  <si>
+    <t>CC 1</t>
+  </si>
+  <si>
+    <t>2.2.2010</t>
+  </si>
+  <si>
+    <t>CC 2</t>
+  </si>
+  <si>
+    <t>2.2.2020</t>
+  </si>
+  <si>
+    <t>CC 3</t>
+  </si>
+  <si>
+    <t>2.2.2030</t>
+  </si>
+  <si>
+    <t>Accrued Construction Costs</t>
+  </si>
+  <si>
+    <t>2.3.3000</t>
+  </si>
+  <si>
+    <t>Buyer Deposits</t>
+  </si>
+  <si>
+    <t>2.4.4000</t>
+  </si>
+  <si>
+    <t>Loan 1</t>
+  </si>
+  <si>
+    <t>2.4.4010</t>
+  </si>
+  <si>
+    <t>Loan 2</t>
+  </si>
+  <si>
+    <t>2.4.4020</t>
+  </si>
+  <si>
+    <t>Loan 3</t>
+  </si>
+  <si>
+    <t>2.5.5000</t>
+  </si>
+  <si>
+    <t>Payroll Liabilities</t>
+  </si>
+  <si>
+    <t>2.6.6000</t>
+  </si>
+  <si>
+    <t>Employment Tax Withholdings</t>
+  </si>
+  <si>
+    <t>3.1.1000</t>
+  </si>
+  <si>
+    <t>Opening Balance Equity</t>
+  </si>
+  <si>
+    <t>3.2.3000</t>
+  </si>
+  <si>
+    <t>Capital Account 1</t>
+  </si>
+  <si>
+    <t>3.2.3010</t>
+  </si>
+  <si>
+    <t>Capital Account 2</t>
+  </si>
+  <si>
+    <t>3.2.3020</t>
+  </si>
+  <si>
+    <t>Distribution Account 1</t>
+  </si>
+  <si>
+    <t>3.2.3030</t>
+  </si>
+  <si>
+    <t>Distribution Account 2</t>
+  </si>
+  <si>
+    <t>3.3.4000</t>
+  </si>
+  <si>
+    <t>Retained Earnings</t>
+  </si>
+  <si>
+    <t>4.1.1000</t>
+  </si>
+  <si>
+    <t>Construction Income</t>
+  </si>
+  <si>
+    <t>5.1.1000</t>
+  </si>
+  <si>
+    <t>COGS - Land</t>
+  </si>
+  <si>
+    <t>5.1.1100</t>
+  </si>
+  <si>
+    <t>COGS - Vertical</t>
+  </si>
+  <si>
+    <t>5.1.1200</t>
+  </si>
+  <si>
+    <t>Cost after sales</t>
+  </si>
+  <si>
+    <t>5.2.2000</t>
+  </si>
+  <si>
+    <t>Bank Fees</t>
+  </si>
+  <si>
+    <t>5.2.2010</t>
+  </si>
+  <si>
+    <t>Interest Expense</t>
+  </si>
+  <si>
+    <t>5.2.2020</t>
+  </si>
+  <si>
+    <t>False Alarms</t>
+  </si>
+  <si>
+    <t>5.2.2030</t>
+  </si>
+  <si>
+    <t>Insurance Expense</t>
+  </si>
+  <si>
+    <t>5.2.2040</t>
+  </si>
+  <si>
+    <t>Legal Fees</t>
+  </si>
+  <si>
+    <t>5.2.2050</t>
+  </si>
+  <si>
+    <t>Property Taxes</t>
+  </si>
+  <si>
+    <t>5.2.2060</t>
+  </si>
+  <si>
+    <t>Professional Fees</t>
+  </si>
+  <si>
+    <t>5.2.2070</t>
+  </si>
+  <si>
+    <t>Insurance Claims</t>
+  </si>
+  <si>
+    <t>5.3.3000</t>
+  </si>
+  <si>
+    <t>Depreciation Expense</t>
+  </si>
+  <si>
+    <t>5.3.3010</t>
+  </si>
+  <si>
+    <t>Petty Cash</t>
+  </si>
+  <si>
+    <t>5.3.3020</t>
+  </si>
+  <si>
+    <t>Auto and Truck Expenses</t>
+  </si>
+  <si>
+    <t>5.3.3040</t>
+  </si>
+  <si>
+    <t>Business License</t>
+  </si>
+  <si>
+    <t>5.3.3050</t>
+  </si>
+  <si>
+    <t>Computer and Internet Expenses</t>
+  </si>
+  <si>
+    <t>5.3.3060</t>
+  </si>
+  <si>
+    <t>Meals and Entertainment</t>
+  </si>
+  <si>
+    <t>5.3.3070</t>
+  </si>
+  <si>
+    <t>Office Expense</t>
+  </si>
+  <si>
+    <t>5.3.3080</t>
+  </si>
+  <si>
+    <t>Subscriptions</t>
+  </si>
+  <si>
+    <t>5.3.3090</t>
+  </si>
+  <si>
+    <t>Telephone Expense</t>
+  </si>
+  <si>
+    <t>5.3.3100</t>
+  </si>
+  <si>
+    <t>Reconciliation Discrepancies</t>
+  </si>
+  <si>
+    <t>5.3.3110</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>5.4.4000</t>
+  </si>
+  <si>
+    <t>State and Federal Taxes</t>
+  </si>
+  <si>
+    <t>5.5.5000</t>
+  </si>
+  <si>
+    <t>Bad Debts</t>
+  </si>
+  <si>
+    <t>5.6.6000</t>
+  </si>
+  <si>
+    <t>Payroll Expenses: Gross Wages</t>
+  </si>
+  <si>
+    <t>5.6.6010</t>
+  </si>
+  <si>
+    <t>Payroll Expenses: Payroll Processing Expense</t>
+  </si>
+  <si>
+    <t>5.6.6020</t>
+  </si>
+  <si>
+    <t>Payroll Expenses: Payroll Taxes and Benefits</t>
+  </si>
+  <si>
+    <t>6.1.1000</t>
+  </si>
+  <si>
+    <t>Charitable Contributions</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>account_id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -454,10 +709,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="4"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -775,7 +1030,7 @@
   <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="45.1640625" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" customWidth="1"/>
@@ -784,8 +1039,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>49</v>
+      <c r="A1" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -794,16 +1049,16 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
@@ -812,109 +1067,109 @@
         <v>6</v>
       </c>
       <c r="J1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="K1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>53</v>
+      <c r="A2" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="H2" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="J2">
         <v>30342</v>
       </c>
       <c r="K2" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>56</v>
+      <c r="A3" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="H3" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="J3">
         <v>30342</v>
       </c>
       <c r="K3" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D4" t="s">
-        <v>68</v>
-      </c>
       <c r="E4" t="b">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="G4" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="J4">
         <v>30328</v>
       </c>
       <c r="K4" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -924,75 +1179,155 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2087A0E-BB58-0C4C-BAF6-1FBB64EB8FEB}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="46.33203125" customWidth="1"/>
+    <col min="2" max="2" width="45.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>1</v>
+      <c r="A2" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>2</v>
+      <c r="A3" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>3</v>
+      <c r="A4" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>4</v>
+      <c r="A5" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>5</v>
+      <c r="A6" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>6</v>
+      <c r="A7" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>7</v>
+      <c r="A8" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1002,71 +1337,836 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7FFABB-7DD7-CF45-A769-F5722E7ACEDD}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="7.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>209</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>51</v>
-      </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D2" s="1" t="s">
-        <v>10</v>
+      <c r="A2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2">
+        <v>100</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D3" s="1" t="s">
-        <v>11</v>
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3">
+        <v>200</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D4" s="1" t="s">
-        <v>12</v>
+      <c r="A4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4">
+        <v>300</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D5" s="1" t="s">
-        <v>13</v>
+      <c r="A5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5">
+        <v>400</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D6" s="1" t="s">
-        <v>14</v>
+      <c r="A6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6">
+        <v>500</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D7" s="1" t="s">
-        <v>15</v>
+      <c r="A7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7">
+        <v>600</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D8" s="1" t="s">
-        <v>16</v>
+      <c r="A8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8">
+        <v>700</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9">
+        <v>800</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10">
+        <v>900</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11">
+        <v>1000</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12">
+        <v>1100</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13">
+        <v>1200</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14">
+        <v>1300</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C15">
+        <v>1400</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16">
+        <v>1500</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17">
+        <v>1600</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C18">
+        <v>1700</v>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19">
+        <v>1800</v>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" t="s">
+        <v>131</v>
+      </c>
+      <c r="C20">
+        <v>1900</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>132</v>
+      </c>
+      <c r="B21" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21">
+        <v>2000</v>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22">
+        <v>2100</v>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23">
+        <v>2200</v>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24">
+        <v>2300</v>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25">
+        <v>2400</v>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>142</v>
+      </c>
+      <c r="B26" t="s">
+        <v>143</v>
+      </c>
+      <c r="C26">
+        <v>2500</v>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" t="s">
+        <v>145</v>
+      </c>
+      <c r="C27">
+        <v>2600</v>
+      </c>
+      <c r="E27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>146</v>
+      </c>
+      <c r="B28" t="s">
+        <v>147</v>
+      </c>
+      <c r="C28">
+        <v>2700</v>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>148</v>
+      </c>
+      <c r="B29" t="s">
+        <v>149</v>
+      </c>
+      <c r="C29">
+        <v>2800</v>
+      </c>
+      <c r="E29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" t="s">
+        <v>151</v>
+      </c>
+      <c r="C30">
+        <v>2900</v>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" t="s">
+        <v>153</v>
+      </c>
+      <c r="C31">
+        <v>3000</v>
+      </c>
+      <c r="E31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32">
+        <v>3100</v>
+      </c>
+      <c r="E32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33" t="s">
+        <v>157</v>
+      </c>
+      <c r="C33">
+        <v>3200</v>
+      </c>
+      <c r="E33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>158</v>
+      </c>
+      <c r="B34" t="s">
+        <v>159</v>
+      </c>
+      <c r="C34">
+        <v>3300</v>
+      </c>
+      <c r="E34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>160</v>
+      </c>
+      <c r="B35" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35">
+        <v>3400</v>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>162</v>
+      </c>
+      <c r="B36" t="s">
+        <v>163</v>
+      </c>
+      <c r="C36">
+        <v>3500</v>
+      </c>
+      <c r="E36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>164</v>
+      </c>
+      <c r="B37" t="s">
+        <v>165</v>
+      </c>
+      <c r="C37">
+        <v>3600</v>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>166</v>
+      </c>
+      <c r="B38" t="s">
+        <v>167</v>
+      </c>
+      <c r="C38">
+        <v>3700</v>
+      </c>
+      <c r="E38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>168</v>
+      </c>
+      <c r="B39" t="s">
+        <v>169</v>
+      </c>
+      <c r="C39">
+        <v>3800</v>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>170</v>
+      </c>
+      <c r="B40" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40">
+        <v>3900</v>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>172</v>
+      </c>
+      <c r="B41" t="s">
+        <v>173</v>
+      </c>
+      <c r="C41">
+        <v>4000</v>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>174</v>
+      </c>
+      <c r="B42" t="s">
+        <v>175</v>
+      </c>
+      <c r="C42">
+        <v>4100</v>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>176</v>
+      </c>
+      <c r="B43" t="s">
+        <v>177</v>
+      </c>
+      <c r="C43">
+        <v>4200</v>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>178</v>
+      </c>
+      <c r="B44" t="s">
+        <v>179</v>
+      </c>
+      <c r="C44">
+        <v>4300</v>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B45" t="s">
+        <v>181</v>
+      </c>
+      <c r="C45">
+        <v>4400</v>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>182</v>
+      </c>
+      <c r="B46" t="s">
+        <v>183</v>
+      </c>
+      <c r="C46">
+        <v>4500</v>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>184</v>
+      </c>
+      <c r="B47" t="s">
+        <v>185</v>
+      </c>
+      <c r="C47">
+        <v>4600</v>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>186</v>
+      </c>
+      <c r="B48" t="s">
+        <v>187</v>
+      </c>
+      <c r="C48">
+        <v>4700</v>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>188</v>
+      </c>
+      <c r="B49" t="s">
+        <v>189</v>
+      </c>
+      <c r="C49">
+        <v>4800</v>
+      </c>
+      <c r="E49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>190</v>
+      </c>
+      <c r="B50" t="s">
+        <v>191</v>
+      </c>
+      <c r="C50">
+        <v>4900</v>
+      </c>
+      <c r="E50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>192</v>
+      </c>
+      <c r="B51" t="s">
+        <v>193</v>
+      </c>
+      <c r="C51">
+        <v>5000</v>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>194</v>
+      </c>
+      <c r="B52" t="s">
+        <v>195</v>
+      </c>
+      <c r="C52">
+        <v>5100</v>
+      </c>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>196</v>
+      </c>
+      <c r="B53" t="s">
+        <v>197</v>
+      </c>
+      <c r="C53">
+        <v>5200</v>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>198</v>
+      </c>
+      <c r="B54" t="s">
+        <v>199</v>
+      </c>
+      <c r="C54">
+        <v>5300</v>
+      </c>
+      <c r="E54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>200</v>
+      </c>
+      <c r="B55" t="s">
+        <v>201</v>
+      </c>
+      <c r="C55">
+        <v>5400</v>
+      </c>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>202</v>
+      </c>
+      <c r="B56" t="s">
+        <v>203</v>
+      </c>
+      <c r="C56">
+        <v>5500</v>
+      </c>
+      <c r="E56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>204</v>
+      </c>
+      <c r="B57" t="s">
+        <v>205</v>
+      </c>
+      <c r="C57">
+        <v>5600</v>
+      </c>
+      <c r="E57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>206</v>
+      </c>
+      <c r="B58" t="s">
+        <v>207</v>
+      </c>
+      <c r="C58">
+        <v>5700</v>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1087,7 +2187,7 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
         <v>5</v>
@@ -1121,46 +2221,46 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" t="s">
         <v>17</v>
       </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" t="s">
-        <v>38</v>
-      </c>
-      <c r="K1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M1" t="s">
-        <v>24</v>
-      </c>
       <c r="N1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1175,34 +2275,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="G1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="H1" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="I1" t="s">
         <v>1</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1234,49 +2334,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" t="s">
-        <v>35</v>
-      </c>
-      <c r="K1" t="s">
-        <v>33</v>
-      </c>
       <c r="L1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="M1" t="s">
         <v>9</v>
       </c>
       <c r="N1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="O1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Postman Tests for GL Admin routes
</commit_message>
<xml_diff>
--- a/test/Assets/Lists.xlsx
+++ b/test/Assets/Lists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ian/Documents/Projects/nap/test/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EFDE32-8A9A-3447-A445-024C539E8FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CD9E42-B7EF-0B42-8D53-F8FA1A446CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="4280" windowWidth="28040" windowHeight="17440" activeTab="3" xr2:uid="{C06FBE5E-17A7-D341-AC99-42140C686358}"/>
+    <workbookView xWindow="4280" yWindow="4280" windowWidth="28040" windowHeight="17440" xr2:uid="{C06FBE5E-17A7-D341-AC99-42140C686358}"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="243">
   <si>
     <t>company</t>
   </si>
@@ -691,6 +691,87 @@
   </si>
   <si>
     <t>inter_company_classification</t>
+  </si>
+  <si>
+    <t>30342</t>
+  </si>
+  <si>
+    <t>30328</t>
+  </si>
+  <si>
+    <t>020</t>
+  </si>
+  <si>
+    <t>Peony Farms</t>
+  </si>
+  <si>
+    <t>100 townhouses in Peony Plantations</t>
+  </si>
+  <si>
+    <t>22-235777</t>
+  </si>
+  <si>
+    <t>1069 Penny Place</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Peony</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>78012</t>
+  </si>
+  <si>
+    <t>030</t>
+  </si>
+  <si>
+    <t>Dahlia</t>
+  </si>
+  <si>
+    <t>40 sindle family homes</t>
+  </si>
+  <si>
+    <t>33-167824</t>
+  </si>
+  <si>
+    <t>2042 Daisy Lane</t>
+  </si>
+  <si>
+    <t>Unit A6</t>
+  </si>
+  <si>
+    <t>Carmel</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>48901</t>
+  </si>
+  <si>
+    <t>040</t>
+  </si>
+  <si>
+    <t>WEG Azalea Heights, LLC</t>
+  </si>
+  <si>
+    <t>25 Townhomes</t>
+  </si>
+  <si>
+    <t>11-229871</t>
+  </si>
+  <si>
+    <t>242 Plaza Lane</t>
+  </si>
+  <si>
+    <t>30319</t>
+  </si>
+  <si>
+    <t>050</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1133,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52E00720-9E0C-5F49-8085-79AD84E3B1F5}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" style="1" customWidth="1"/>
@@ -1099,7 +1180,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>39</v>
       </c>
       <c r="B2" t="s">
@@ -1123,15 +1204,15 @@
       <c r="I2" t="s">
         <v>50</v>
       </c>
-      <c r="J2">
-        <v>30342</v>
+      <c r="J2" t="s">
+        <v>216</v>
       </c>
       <c r="K2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>42</v>
       </c>
       <c r="B3" t="s">
@@ -1155,15 +1236,15 @@
       <c r="I3" t="s">
         <v>50</v>
       </c>
-      <c r="J3">
-        <v>30342</v>
+      <c r="J3" t="s">
+        <v>216</v>
       </c>
       <c r="K3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>40</v>
       </c>
       <c r="B4" t="s">
@@ -1190,10 +1271,150 @@
       <c r="I4" t="s">
         <v>50</v>
       </c>
-      <c r="J4">
-        <v>30328</v>
+      <c r="J4" t="s">
+        <v>217</v>
       </c>
       <c r="K4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B5" t="s">
+        <v>219</v>
+      </c>
+      <c r="C5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D5" t="s">
+        <v>221</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>222</v>
+      </c>
+      <c r="G5" t="s">
+        <v>223</v>
+      </c>
+      <c r="H5" t="s">
+        <v>224</v>
+      </c>
+      <c r="I5" t="s">
+        <v>225</v>
+      </c>
+      <c r="J5" t="s">
+        <v>226</v>
+      </c>
+      <c r="K5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B6" t="s">
+        <v>228</v>
+      </c>
+      <c r="C6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>231</v>
+      </c>
+      <c r="G6" t="s">
+        <v>232</v>
+      </c>
+      <c r="H6" t="s">
+        <v>233</v>
+      </c>
+      <c r="I6" t="s">
+        <v>234</v>
+      </c>
+      <c r="J6" t="s">
+        <v>235</v>
+      </c>
+      <c r="K6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D7" t="s">
+        <v>239</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
+        <v>240</v>
+      </c>
+      <c r="G7" t="s">
+        <v>223</v>
+      </c>
+      <c r="H7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" t="s">
+        <v>241</v>
+      </c>
+      <c r="K7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" t="s">
+        <v>238</v>
+      </c>
+      <c r="D8" t="s">
+        <v>239</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>240</v>
+      </c>
+      <c r="G8" t="s">
+        <v>223</v>
+      </c>
+      <c r="H8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J8" t="s">
+        <v>241</v>
+      </c>
+      <c r="K8" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>